<commit_message>
Added core hours to analysis
</commit_message>
<xml_diff>
--- a/mesh_study_results.xlsx
+++ b/mesh_study_results.xlsx
@@ -2432,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2445,6 +2445,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2480,20 +2481,25 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Core-Hours</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Cell Count (M)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Solve Time / Iteration (s) vs 30mm (%)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Total Wall Time (min) vs 30mm (%)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Cell Count (M) vs 30mm (%)</t>
         </is>
@@ -2518,14 +2524,17 @@
         <v>92.63333333333334</v>
       </c>
       <c r="F2" t="n">
-        <v>3.8128</v>
+        <v>3.812799997106195</v>
       </c>
       <c r="G2" t="n">
+        <v>220.7761111049331</v>
+      </c>
+      <c r="H2" t="n">
         <v>39.094249</v>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2546,18 +2555,21 @@
         <v>85.03333333333333</v>
       </c>
       <c r="F3" t="n">
-        <v>3.4544</v>
+        <v>3.454399996306747</v>
       </c>
       <c r="G3" t="n">
+        <v>202.6627776825917</v>
+      </c>
+      <c r="H3" t="n">
         <v>37.490479</v>
       </c>
-      <c r="H3" t="n">
-        <v>-9.399916072177927</v>
-      </c>
       <c r="I3" t="n">
+        <v>-9.399916100279651</v>
+      </c>
+      <c r="J3" t="n">
         <v>-8.204390068369925</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>-4.102316941809005</v>
       </c>
     </row>
@@ -2580,18 +2592,21 @@
         <v>67.26666666666667</v>
       </c>
       <c r="F4" t="n">
-        <v>3.7040704070407</v>
+        <v>3.704070406366545</v>
       </c>
       <c r="G4" t="n">
+        <v>160.3188890086021</v>
+      </c>
+      <c r="H4" t="n">
         <v>36.840164</v>
       </c>
-      <c r="H4" t="n">
-        <v>-2.851699353737415</v>
-      </c>
       <c r="I4" t="n">
+        <v>-2.851699297685997</v>
+      </c>
+      <c r="J4" t="n">
         <v>-27.38395106153293</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>-5.765771328667796</v>
       </c>
     </row>
@@ -2614,18 +2629,21 @@
         <v>85.01666666666667</v>
       </c>
       <c r="F5" t="n">
-        <v>3.4664</v>
+        <v>3.46640000263229</v>
       </c>
       <c r="G5" t="n">
+        <v>202.6230557257659</v>
+      </c>
+      <c r="H5" t="n">
         <v>35.731616</v>
       </c>
-      <c r="H5" t="n">
-        <v>-9.085186739404113</v>
-      </c>
       <c r="I5" t="n">
+        <v>-9.085186601364144</v>
+      </c>
+      <c r="J5" t="n">
         <v>-8.222382151853193</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>-8.601349523301996</v>
       </c>
     </row>
@@ -2648,18 +2666,21 @@
         <v>79.78333333333333</v>
       </c>
       <c r="F6" t="n">
-        <v>3.2224000008</v>
+        <v>3.222400002423674</v>
       </c>
       <c r="G6" t="n">
+        <v>190.1502778041176</v>
+      </c>
+      <c r="H6" t="n">
         <v>34.741504</v>
       </c>
-      <c r="H6" t="n">
-        <v>-15.48468315148972</v>
-      </c>
       <c r="I6" t="n">
+        <v>-15.4846830447602</v>
+      </c>
+      <c r="J6" t="n">
         <v>-13.87189636559915</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>-11.13397778788384</v>
       </c>
     </row>

</xml_diff>